<commit_message>
Solucion a plan de vulnerabilidades
</commit_message>
<xml_diff>
--- a/Documentacion/Gantt Proyecto Integrador Sistema Inscripciones UTSC.xlsx
+++ b/Documentacion/Gantt Proyecto Integrador Sistema Inscripciones UTSC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Froylan Grimaldo\Desktop\utsc_inscripciones\Documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Froylan Grimaldo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560C872E-7E56-407B-9924-BEE86DF8DA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F328C831-91EE-47F6-8452-FB77274FA34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,12 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="53">
   <si>
     <t>DIAGRAMA DE GANTT — PROYECTO INTEGRADOR 2026: SISTEMA DE INSCRIPCIONES UTSC (PÁGINA WEB Y APP MÓVIL)</t>
   </si>
   <si>
-    <t>Universidad Tecnológica Santa Catarina  |  Septiembre – Noviembre 2026  |  Corte de avance: 20/10/2026</t>
+    <t>Universidad Tecnológica Santa Catarina  |  Septiembre – Noviembre 2026  |  Corte de avance: 26/10/2026</t>
   </si>
   <si>
     <t>#</t>
@@ -144,7 +144,7 @@
     <t>Desarrollo backend y API REST (Flask, JWT)</t>
   </si>
   <si>
-    <t>Completada con +1 semana de desviación: se agregaron endpoints de dashboard, reportes Excel y motivo de rechazo (requerimiento nuevo). Falta publicarlos en Render.</t>
+    <t>Completada con +1 semana de desviación: se agregaron endpoints de dashboard, reportes Excel y motivo de rechazo (requerimiento nuevo). Ya publicados en Render.</t>
   </si>
   <si>
     <t>Desarrollo web (frontend)</t>
@@ -156,31 +156,31 @@
     <t>Desarrollo app móvil (Flutter)</t>
   </si>
   <si>
-    <t>En retraso (≈1 semana): dashboard y reportes de la app aún no se prueban contra el servidor publicado y el envío de inscripción móvil sigue simulado. Pendiente conectarlo al servidor.</t>
+    <t>Completada con ≈1 semana de retraso (plan: 18/10; terminada en S8) porque el dashboard y los reportes dependían de publicar el backend. Por confirmar: el envío de inscripción móvil estaba simulado.</t>
   </si>
   <si>
     <t>Nuevas funciones: dashboard, reportes, motivo de rechazo y edad</t>
   </si>
   <si>
-    <t>Requerimiento adicional solicitado el 11/10; no estaba en el plan original. Código y pruebas de servidor listos (70 verificaciones). Falta probarlo en producción.</t>
+    <t>Completada en la fecha planeada (25/10) y publicada en Render. Fue un requerimiento adicional solicitado el 11/10; no estaba en el plan original.</t>
   </si>
   <si>
     <t>Seguridad y corrección de vulnerabilidades</t>
   </si>
   <si>
-    <t>Plan de 17 vulnerabilidades elaborado el 20/10. Correcciones pendientes: almacenamiento seguro del token, CSRF, límite de intentos, ofuscación y respaldo de Android.</t>
+    <t>En proceso: plan de 17 vulnerabilidades elaborado el 20/10 y avance en S8. Pendiente el resto de correcciones (almacenamiento seguro del token, CSRF, límite de intentos, ofuscación, respaldo de Android).</t>
   </si>
   <si>
     <t>Integración y pruebas</t>
   </si>
   <si>
-    <t>Pruebas automatizadas (40 casos), Postman y regresión hechas en septiembre. Pendiente repetirlas con las funciones nuevas y las correcciones de seguridad.</t>
+    <t>Pruebas automatizadas (40 casos), Postman y regresión hechas en septiembre; en S8 se avanzó con las funciones nuevas. Pendiente repetirlas tras las correcciones de seguridad.</t>
   </si>
   <si>
     <t>Documentación</t>
   </si>
   <si>
-    <t>Plan de pruebas, documentación técnica y manual de usuario entregados. Pendiente actualizarlos con dashboard, reportes, motivo de rechazo y seguridad.</t>
+    <t>Plan de pruebas, documentación técnica y manual de usuario entregados; en S8 se avanzó en su actualización. Pendiente incluir dashboard, reportes, motivo de rechazo y seguridad, y subir el Gantt al repositorio.</t>
   </si>
   <si>
     <t>Presentación final</t>
@@ -204,7 +204,7 @@
     <t>Semana completada (avance real)</t>
   </si>
   <si>
-    <t>Semana actual (corte 20/10/2026)</t>
+    <t>Semana actual (corte 26/10/2026)</t>
   </si>
   <si>
     <t>Cómo registrar el avance cada semana: escribe ✔ en la celda de la semana terminada; se pinta de azul y el % de avance y el estado se actualizan solos. Anota en Observaciones cualquier desviación.</t>
@@ -900,10 +900,10 @@
       <c r="K4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="M4" s="8" t="s">
         <v>14</v>
       </c>
       <c r="N4" s="7" t="s">
@@ -1176,7 +1176,9 @@
       <c r="K10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="L10" s="13"/>
+      <c r="L10" s="12" t="s">
+        <v>23</v>
+      </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
       <c r="O10" s="13"/>

</xml_diff>